<commit_message>
protecting sheet with password
</commit_message>
<xml_diff>
--- a/Kengen_Generation_Mix/Kengen_Generation_Mix_Analysis.xlsx
+++ b/Kengen_Generation_Mix/Kengen_Generation_Mix_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d40da75d89d0665/Desktop/EXCEL PROJECTS/Excel_Projects/Kengen_Generation_Mix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="14_{55C727FD-2C7B-4B82-B271-FE598888B0EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8674A82D-9311-4080-A5A6-7D667F441CFA}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="14_{55C727FD-2C7B-4B82-B271-FE598888B0EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4279CA51-D13A-41C8-AEB9-CB19820E14FB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="6" xr2:uid="{3F756AD5-448C-4C5A-8A2B-EC70492F2E8F}"/>
   </bookViews>
@@ -5866,7 +5866,7 @@
     </row>
     <row r="18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="dUAKqWI5agApvfG63RSqyLdSMDU/Evv/Cj5PmlrYeTEIthxlKFpHS8RoiX9kHONh/8IJnlKReniWmowELVVeVg==" saltValue="QH0O/vCbdVioy1I9HR/ATg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>